<commit_message>
Aalborg results are reorganized
</commit_message>
<xml_diff>
--- a/AalborgResults/Two_Objectives/without PP cofiguration/Pareto-front-0_20140604SM_MCed.xlsx
+++ b/AalborgResults/Two_Objectives/without PP cofiguration/Pareto-front-0_20140604SM_MCed.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahbub\Documents\GitHub\EnergyPLANDomainKnowledgeEAStep1\AalborgResults\Two_Objectives\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahbub\Documents\GitHub\EnergyPLANDomainKnowledgeEAStep1\AalborgResults\Two_Objectives\without PP cofiguration\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20460" windowHeight="7830"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -412,14 +412,14 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -502,6 +502,10 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -1142,6 +1146,8 @@
             </a:ln>
           </c:spPr>
           <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
                 <a:srgbClr val="92D050"/>
@@ -1187,11 +1193,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="312596760"/>
-        <c:axId val="312599504"/>
+        <c:axId val="306311280"/>
+        <c:axId val="324682792"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="312596760"/>
+        <c:axId val="306311280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -1210,7 +1216,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="it-IT"/>
-                  <a:t>CO2 emission in Mton</a:t>
+                  <a:t>CO2 emission [Mt]</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -1222,14 +1228,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="312599504"/>
+        <c:crossAx val="324682792"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
         <c:minorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="312599504"/>
+        <c:axId val="324682792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="2000"/>
@@ -1261,7 +1267,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="312596760"/>
+        <c:crossAx val="306311280"/>
         <c:crossesAt val="0"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1000"/>
@@ -1329,7 +1335,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>PP with respect</a:t>
+              <a:t>PP capacity with respect</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
@@ -1351,21 +1357,17 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$F$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>PP_C</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>PP</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -1994,11 +1996,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="335033704"/>
-        <c:axId val="335037624"/>
+        <c:axId val="324680832"/>
+        <c:axId val="324683184"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="335033704"/>
+        <c:axId val="324680832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -2008,15 +2010,19 @@
         <c:axPos val="b"/>
         <c:title>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$Z$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>CO2 Emission</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>CO2 Emission [Mt]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
           </c:tx>
           <c:layout/>
           <c:overlay val="0"/>
@@ -2025,13 +2031,13 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335037624"/>
+        <c:crossAx val="324683184"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:minorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="335037624"/>
+        <c:axId val="324683184"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2040,34 +2046,28 @@
         <c:majorGridlines/>
         <c:title>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$AA$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Annual cost </c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Capacity [MW]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
           </c:tx>
           <c:layout/>
           <c:overlay val="0"/>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" vert="horz"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr/>
-              </a:pPr>
-              <a:endParaRPr lang="it-IT"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="0" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335033704"/>
+        <c:crossAx val="324680832"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2113,13 +2113,14 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Pareto-optimal</a:t>
+              <a:rPr lang="en-US" sz="1800" b="1" i="0" baseline="0">
+                <a:effectLst/>
+              </a:rPr>
+              <a:t>wind, off-shore and total wind capacity with respect to CO2 emission</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Front</a:t>
-            </a:r>
+            <a:endParaRPr lang="it-IT">
+              <a:effectLst/>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -2146,21 +2147,17 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$H$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>wind_C</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Onshore Wind</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -2785,21 +2782,17 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$J$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Off-Shore Wind_C</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Offshore wind</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -3428,8 +3421,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="335039192"/>
-        <c:axId val="335039584"/>
+        <c:axId val="324681224"/>
+        <c:axId val="324681616"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -3453,6 +3446,10 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -4081,11 +4078,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="335035272"/>
-        <c:axId val="335031744"/>
+        <c:axId val="324682400"/>
+        <c:axId val="324683576"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="335039192"/>
+        <c:axId val="324681224"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -4095,15 +4092,19 @@
         <c:axPos val="b"/>
         <c:title>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$Z$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>CO2 Emission</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>CO2 Emission [Mt]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
           </c:tx>
           <c:layout/>
           <c:overlay val="0"/>
@@ -4112,14 +4113,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335039584"/>
+        <c:crossAx val="324681616"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
         <c:minorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="335039584"/>
+        <c:axId val="324681616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4128,39 +4129,38 @@
         <c:majorGridlines/>
         <c:title>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$AA$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Annual cost </c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Capacity</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> [MW]</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
           </c:tx>
           <c:layout/>
           <c:overlay val="0"/>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" vert="horz"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr/>
-              </a:pPr>
-              <a:endParaRPr lang="it-IT"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="0" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335039192"/>
+        <c:crossAx val="324681224"/>
         <c:crossesAt val="-0.60000000000000009"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="335031744"/>
+        <c:axId val="324683576"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4170,12 +4170,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335035272"/>
+        <c:crossAx val="324682400"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="335035272"/>
+        <c:axId val="324682400"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4185,7 +4185,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335031744"/>
+        <c:crossAx val="324683576"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4251,7 +4251,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>CHP and HP with respect to CO2</a:t>
+              <a:t>CHP and HP capacity with respect to CO2</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" baseline="0"/>
           </a:p>
@@ -4270,21 +4270,17 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$D$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>HP3_C</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>HP</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -4909,21 +4905,17 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>CHP3_C</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>CHP</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="4"/>
+          </c:marker>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$Z$5:$Z$104</c:f>
@@ -5552,11 +5544,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="335041936"/>
-        <c:axId val="335034880"/>
+        <c:axId val="324679656"/>
+        <c:axId val="324677304"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="335041936"/>
+        <c:axId val="324679656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.60000000000000009"/>
@@ -5575,7 +5567,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>CO2 Emission in Mton</a:t>
+                  <a:t>CO2 Emission [Mt]</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -5587,14 +5579,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335034880"/>
+        <c:crossAx val="324677304"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
         <c:minorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="335034880"/>
+        <c:axId val="324677304"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5612,7 +5604,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="it-IT"/>
-                  <a:t>Capacity in MW</a:t>
+                  <a:t>Capacity [MW]</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -5624,7 +5616,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="335041936"/>
+        <c:crossAx val="324679656"/>
         <c:crossesAt val="-1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5718,10 +5710,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>44</xdr:col>
-      <xdr:colOff>609599</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>280147</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6398,41 +6390,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="D1" s="39" t="s">
+      <c r="D1" s="37" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:47" ht="21" x14ac:dyDescent="0.35">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
-      <c r="O2" s="37" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="O2" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="P2" s="37"/>
-      <c r="Q2" s="37"/>
-      <c r="R2" s="37"/>
-      <c r="S2" s="37"/>
-      <c r="T2" s="37"/>
-      <c r="U2" s="37"/>
-      <c r="V2" s="37"/>
-      <c r="W2" s="37"/>
-      <c r="X2" s="37"/>
-      <c r="Z2" s="37" t="s">
+      <c r="P2" s="38"/>
+      <c r="Q2" s="38"/>
+      <c r="R2" s="38"/>
+      <c r="S2" s="38"/>
+      <c r="T2" s="38"/>
+      <c r="U2" s="38"/>
+      <c r="V2" s="38"/>
+      <c r="W2" s="38"/>
+      <c r="X2" s="38"/>
+      <c r="Z2" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="AA2" s="37"/>
+      <c r="AA2" s="38"/>
     </row>
     <row r="3" spans="1:47" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -9459,18 +9451,18 @@
         <f t="shared" si="7"/>
         <v>2222</v>
       </c>
-      <c r="AE35" s="38" t="s">
+      <c r="AE35" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="AF35" s="38"/>
-      <c r="AG35" s="38"/>
-      <c r="AH35" s="38"/>
-      <c r="AI35" s="38"/>
-      <c r="AJ35" s="38"/>
-      <c r="AK35" s="38"/>
-      <c r="AL35" s="38"/>
-      <c r="AM35" s="38"/>
-      <c r="AN35" s="38"/>
+      <c r="AF35" s="39"/>
+      <c r="AG35" s="39"/>
+      <c r="AH35" s="39"/>
+      <c r="AI35" s="39"/>
+      <c r="AJ35" s="39"/>
+      <c r="AK35" s="39"/>
+      <c r="AL35" s="39"/>
+      <c r="AM35" s="39"/>
+      <c r="AN35" s="39"/>
       <c r="AU35" s="12"/>
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.25">

</xml_diff>